<commit_message>
feat: 9 StatCan publication fixture workbooks covering T101/C101 rules
</commit_message>
<xml_diff>
--- a/tests/fixtures/test_cases/bilingual_gdp.xlsx
+++ b/tests/fixtures/test_cases/bilingual_gdp.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="tbl1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="tbl1_fr" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,123 +413,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Industry / Industrie</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>GDP (billions)</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Share (%)</t>
+          <t>GDP / PIB</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>All industries</t>
+          <t>Goods / Biens</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2150.5</v>
-      </c>
-      <c r="C2" t="n">
-        <v>100</v>
+        <v>680.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Goods-producing</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>620.8</v>
-      </c>
-      <c r="C3" t="n">
-        <v>28.9</v>
+        <v>1770.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Source: Statistics Canada, GDP.</t>
-        </is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2450.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>x confidential</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Secteur</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>PIB (milliards)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ensemble des industries</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2150.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Biens</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>620.8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Source : Statistique Canada, PIB.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>x confidentiel</t>
+          <t>Source: Statistics Canada</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>..</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>not available</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[verified] release-gate validator demo fixtures and local LLM mode
</commit_message>
<xml_diff>
--- a/tests/fixtures/test_cases/bilingual_gdp.xlsx
+++ b/tests/fixtures/test_cases/bilingual_gdp.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="tbl1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="tbl1_fr" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,72 +414,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Industry / Industrie</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>GDP / PIB</t>
+          <t>GDP (billions)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Share (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Goods / Biens</t>
+          <t>All industries</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>680.2</v>
+        <v>2150.5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Services</t>
+          <t>Goods-producing</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1770.3</v>
+        <v>620.8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>28.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2450.5</v>
+          <t>Source: Statistics Canada, GDP.</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Source: Statistics Canada</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>..</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>not available</t>
+          <t>x confidential</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Secteur</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>PIB (milliards)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ensemble des industries</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2150.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Biens</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>620.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Source : Statistique Canada, PIB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>x confidentiel</t>
         </is>
       </c>
     </row>

</xml_diff>